<commit_message>
feat(milestone-3): complete coalesce logic, delta dataset, and docs
- update README.md to document milestone 3 at 67% progress

- add verification screenshots for coalesce configuration and delta transform

- update dataset with modified and inserted employee records

- update screenshot inventory in .gitkeep
</commit_message>
<xml_diff>
--- a/dataset/Sample Spreadsheet.xlsx
+++ b/dataset/Sample Spreadsheet.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Naan_Mudhalvan\dataset\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6189B0-C24A-49C7-B5B1-CA67A3F116E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="68">
   <si>
     <t>Employee ID</t>
   </si>
@@ -34,9 +43,6 @@
     <t>SB-0004</t>
   </si>
   <si>
-    <t>Ajay</t>
-  </si>
-  <si>
     <t>kumar</t>
   </si>
   <si>
@@ -58,9 +64,6 @@
     <t>V</t>
   </si>
   <si>
-    <t>test10@gmail.com</t>
-  </si>
-  <si>
     <t>Risk &amp; Compliance</t>
   </si>
   <si>
@@ -191,22 +194,81 @@
   </si>
   <si>
     <t>Kochi</t>
+  </si>
+  <si>
+    <t>test18@gmail.com</t>
+  </si>
+  <si>
+    <t>Ajay Kumar</t>
+  </si>
+  <si>
+    <t>SB-0011</t>
+  </si>
+  <si>
+    <t>Suresh</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>suresh.k@testbank.com</t>
+  </si>
+  <si>
+    <t>SB-0012</t>
+  </si>
+  <si>
+    <t>Meena</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>meena.r@testbank.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -215,40 +277,71 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -438,21 +531,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="4" max="4" width="22.25"/>
-    <col customWidth="1" min="5" max="5" width="17.38"/>
+    <col min="4" max="4" width="22.28515625" customWidth="1"/>
+    <col min="5" max="5" width="17.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,207 +568,265 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="D7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E7" s="1" t="s">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="E8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="1" t="s">
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="B9" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C10" s="1" t="s">
+    </row>
+    <row r="11" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>59</v>
-      </c>
+      <c r="F12" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G14" s="6"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{959696D0-5ED9-42F0-9CE1-2E9E86AB69C5}"/>
+    <hyperlink ref="D2" r:id="rId2" xr:uid="{13CC5BD6-ECE5-4485-80C0-BFA96654530C}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{AA485E3B-31D1-448B-8490-EBBF0590ADE2}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{0E90F009-2044-474F-AFAC-66CFF0BDF295}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{B176C637-F8CC-43F9-BF79-EB1DD607DAE6}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{B727E3DB-3023-4810-99EC-C6DB9FC52568}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{06430DE2-7504-4690-A1D9-641CD8F682EA}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{D971EE85-939B-43A0-A7BF-C39B5D3036B9}"/>
+    <hyperlink ref="D10" r:id="rId9" xr:uid="{16A42E02-08C6-4EF4-A426-7B334CDA8472}"/>
+    <hyperlink ref="D11" r:id="rId10" xr:uid="{585D244F-5F9E-467D-A5DF-3A0027C50F08}"/>
+    <hyperlink ref="D12" r:id="rId11" xr:uid="{10CB4E6C-0BE5-4381-A5CD-96B5654C3AEB}"/>
+    <hyperlink ref="D13" r:id="rId12" xr:uid="{69972A4B-F088-4B72-9663-257B5A151419}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>